<commit_message>
Update build order and rest screenshot
</commit_message>
<xml_diff>
--- a/docs/Severance Monsters.xlsx
+++ b/docs/Severance Monsters.xlsx
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Balance Log'!$A$4:$G$30</definedName>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Build Order'!$A$4:$H$19</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Build Order'!$A$4:$H$20</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="821" uniqueCount="468">
   <si>
     <t xml:space="preserve">Severance - Monster Stats</t>
   </si>
@@ -831,6 +831,12 @@
     <t xml:space="preserve">Done</t>
   </si>
   <si>
+    <t xml:space="preserve">Automated tests (pytest)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 tests: damage, blocking, healing, level-up stats, ability unlock, cooldowns. Run with: pytest -v</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mana bar</t>
   </si>
   <si>
@@ -840,7 +846,7 @@
     <t xml:space="preserve">Sorcerer class + Mana Tide</t>
   </si>
   <si>
-    <t xml:space="preserve">Add to class select</t>
+    <t xml:space="preserve">Add to class select. Add tests: can't cast without mana, regen caps at max</t>
   </si>
   <si>
     <t xml:space="preserve">Sorcerer balance sims</t>
@@ -900,9 +906,6 @@
     <t xml:space="preserve">You (mechanic) + me (stats)</t>
   </si>
   <si>
-    <t xml:space="preserve">9</t>
-  </si>
-  <si>
     <t xml:space="preserve">Boss adds enemies to the fight mid-battle</t>
   </si>
   <si>
@@ -921,7 +924,7 @@
     <t xml:space="preserve">Outpost</t>
   </si>
   <si>
-    <t xml:space="preserve">11</t>
+    <t xml:space="preserve">12</t>
   </si>
   <si>
     <t xml:space="preserve">Enemies/bosses drop gold, spend at a shop between dungeons (e.g. mana potions)</t>
@@ -1615,7 +1618,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="47">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1720,18 +1723,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1748,12 +1739,20 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -4151,33 +4150,33 @@
   <dimension ref="A1:M54"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="32"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="26" t="s">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
         <v>130</v>
       </c>
     </row>
@@ -4222,172 +4221,172 @@
         <v>141</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29" t="n">
+    <row r="6" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="26" t="s">
         <v>142</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D6" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="E6" s="29" t="s">
+      <c r="E6" s="26" t="s">
         <v>144</v>
       </c>
-      <c r="F6" s="29" t="s">
+      <c r="F6" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="G6" s="29" t="s">
+      <c r="G6" s="26" t="s">
         <v>146</v>
       </c>
-      <c r="H6" s="29" t="s">
+      <c r="H6" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="29" t="s">
+      <c r="I6" s="26" t="s">
         <v>147</v>
       </c>
-      <c r="J6" s="29" t="s">
+      <c r="J6" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="K6" s="30" t="s">
+      <c r="K6" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="L6" s="29" t="s">
+      <c r="L6" s="26" t="s">
         <v>150</v>
       </c>
-      <c r="M6" s="29" t="s">
+      <c r="M6" s="26" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="n">
+    <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="26" t="s">
         <v>152</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D7" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="E7" s="29" t="s">
+      <c r="E7" s="26" t="s">
         <v>154</v>
       </c>
-      <c r="F7" s="29" t="s">
+      <c r="F7" s="26" t="s">
         <v>155</v>
       </c>
-      <c r="G7" s="29" t="s">
+      <c r="G7" s="26" t="s">
         <v>156</v>
       </c>
-      <c r="H7" s="29" t="s">
+      <c r="H7" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="I7" s="29" t="s">
+      <c r="I7" s="26" t="s">
         <v>158</v>
       </c>
-      <c r="J7" s="29" t="s">
+      <c r="J7" s="26" t="s">
         <v>159</v>
       </c>
-      <c r="K7" s="30" t="s">
+      <c r="K7" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="L7" s="29" t="s">
+      <c r="L7" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="M7" s="29" t="s">
+      <c r="M7" s="26" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29" t="n">
+    <row r="8" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="26" t="s">
         <v>162</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="D8" s="29" t="s">
+      <c r="D8" s="26" t="s">
         <v>164</v>
       </c>
-      <c r="E8" s="29" t="s">
+      <c r="E8" s="26" t="s">
         <v>165</v>
       </c>
-      <c r="F8" s="29" t="s">
+      <c r="F8" s="26" t="s">
         <v>166</v>
       </c>
-      <c r="G8" s="29" t="s">
+      <c r="G8" s="26" t="s">
         <v>167</v>
       </c>
-      <c r="H8" s="29" t="s">
+      <c r="H8" s="26" t="s">
         <v>168</v>
       </c>
-      <c r="I8" s="29" t="s">
+      <c r="I8" s="26" t="s">
         <v>169</v>
       </c>
-      <c r="J8" s="29" t="s">
+      <c r="J8" s="26" t="s">
         <v>170</v>
       </c>
-      <c r="K8" s="31" t="s">
+      <c r="K8" s="28" t="s">
         <v>171</v>
       </c>
-      <c r="L8" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="M8" s="29" t="s">
+      <c r="L8" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="M8" s="26" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="29" t="s">
+    <row r="9" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="26" t="s">
         <v>173</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="26" t="s">
         <v>174</v>
       </c>
-      <c r="D9" s="29" t="s">
+      <c r="D9" s="26" t="s">
         <v>175</v>
       </c>
-      <c r="E9" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" s="29" t="s">
+      <c r="E9" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" s="26" t="s">
         <v>176</v>
       </c>
-      <c r="H9" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="I9" s="29" t="s">
+      <c r="H9" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9" s="26" t="s">
         <v>177</v>
       </c>
-      <c r="J9" s="29" t="s">
+      <c r="J9" s="26" t="s">
         <v>178</v>
       </c>
-      <c r="K9" s="31" t="s">
+      <c r="K9" s="28" t="s">
         <v>171</v>
       </c>
-      <c r="L9" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="M9" s="29" t="s">
+      <c r="L9" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="M9" s="26" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="19" t="s">
         <v>180</v>
       </c>
     </row>
@@ -4421,508 +4420,508 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29" t="n">
+      <c r="A13" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="26" t="s">
         <v>186</v>
       </c>
-      <c r="D13" s="29" t="s">
+      <c r="D13" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="29" t="s">
+      <c r="E13" s="26" t="s">
         <v>187</v>
       </c>
-      <c r="F13" s="29" t="s">
+      <c r="F13" s="26" t="s">
         <v>188</v>
       </c>
-      <c r="G13" s="29" t="s">
+      <c r="G13" s="26" t="s">
         <v>189</v>
       </c>
-      <c r="H13" s="29"/>
-      <c r="I13" s="29"/>
-      <c r="J13" s="29"/>
-      <c r="K13" s="32" t="s">
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="26"/>
+      <c r="K13" s="29" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29" t="n">
+      <c r="A14" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="B14" s="29" t="s">
+      <c r="B14" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="26" t="s">
         <v>186</v>
       </c>
-      <c r="D14" s="29" t="s">
+      <c r="D14" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="E14" s="29" t="s">
+      <c r="E14" s="26" t="s">
         <v>191</v>
       </c>
-      <c r="F14" s="29" t="s">
+      <c r="F14" s="26" t="s">
         <v>192</v>
       </c>
-      <c r="G14" s="29" t="s">
+      <c r="G14" s="26" t="s">
         <v>193</v>
       </c>
-      <c r="H14" s="29"/>
-      <c r="I14" s="29"/>
-      <c r="J14" s="29"/>
-      <c r="K14" s="32" t="s">
+      <c r="H14" s="26"/>
+      <c r="I14" s="26"/>
+      <c r="J14" s="26"/>
+      <c r="K14" s="29" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="29" t="n">
+    <row r="15" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="B15" s="29" t="s">
+      <c r="B15" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="29" t="s">
+      <c r="C15" s="26" t="s">
         <v>186</v>
       </c>
-      <c r="D15" s="29" t="s">
+      <c r="D15" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="29" t="s">
+      <c r="E15" s="26" t="s">
         <v>194</v>
       </c>
-      <c r="F15" s="29" t="s">
+      <c r="F15" s="26" t="s">
         <v>195</v>
       </c>
-      <c r="G15" s="29" t="s">
+      <c r="G15" s="26" t="s">
         <v>196</v>
       </c>
-      <c r="H15" s="29"/>
-      <c r="I15" s="29"/>
-      <c r="J15" s="29"/>
-      <c r="K15" s="32" t="s">
+      <c r="H15" s="26"/>
+      <c r="I15" s="26"/>
+      <c r="J15" s="26"/>
+      <c r="K15" s="29" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="29" t="n">
+    <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="29" t="s">
+      <c r="C16" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="29" t="s">
+      <c r="D16" s="26" t="s">
         <v>197</v>
       </c>
-      <c r="E16" s="29" t="s">
+      <c r="E16" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="F16" s="29" t="s">
+      <c r="F16" s="26" t="s">
         <v>198</v>
       </c>
-      <c r="G16" s="29" t="s">
+      <c r="G16" s="26" t="s">
         <v>199</v>
       </c>
-      <c r="H16" s="29"/>
-      <c r="I16" s="29"/>
-      <c r="J16" s="29"/>
-      <c r="K16" s="32" t="s">
+      <c r="H16" s="26"/>
+      <c r="I16" s="26"/>
+      <c r="J16" s="26"/>
+      <c r="K16" s="29" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="29" t="n">
+    <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B17" s="29" t="s">
+      <c r="B17" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="C17" s="26" t="s">
         <v>200</v>
       </c>
-      <c r="D17" s="29" t="s">
+      <c r="D17" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="29" t="s">
+      <c r="E17" s="26" t="s">
         <v>201</v>
       </c>
-      <c r="F17" s="29" t="s">
+      <c r="F17" s="26" t="s">
         <v>202</v>
       </c>
-      <c r="G17" s="29"/>
-      <c r="H17" s="29"/>
-      <c r="I17" s="29"/>
-      <c r="J17" s="29"/>
-      <c r="K17" s="32" t="s">
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="26"/>
+      <c r="J17" s="26"/>
+      <c r="K17" s="29" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29" t="n">
+    <row r="18" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C18" s="26" t="s">
         <v>200</v>
       </c>
-      <c r="D18" s="29" t="s">
+      <c r="D18" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="E18" s="29" t="s">
+      <c r="E18" s="26" t="s">
         <v>203</v>
       </c>
-      <c r="F18" s="29" t="s">
+      <c r="F18" s="26" t="s">
         <v>204</v>
       </c>
-      <c r="G18" s="29"/>
-      <c r="H18" s="29"/>
-      <c r="I18" s="29"/>
-      <c r="J18" s="29"/>
-      <c r="K18" s="32" t="s">
+      <c r="G18" s="26"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="26"/>
+      <c r="J18" s="26"/>
+      <c r="K18" s="29" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="29" t="n">
+    <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B19" s="29" t="s">
+      <c r="B19" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="29" t="s">
+      <c r="C19" s="26" t="s">
         <v>200</v>
       </c>
-      <c r="D19" s="29" t="s">
+      <c r="D19" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="29" t="s">
+      <c r="E19" s="26" t="s">
         <v>205</v>
       </c>
-      <c r="F19" s="29" t="s">
+      <c r="F19" s="26" t="s">
         <v>204</v>
       </c>
-      <c r="G19" s="29" t="s">
+      <c r="G19" s="26" t="s">
         <v>206</v>
       </c>
-      <c r="H19" s="29"/>
-      <c r="I19" s="29"/>
-      <c r="J19" s="29"/>
-      <c r="K19" s="32" t="s">
+      <c r="H19" s="26"/>
+      <c r="I19" s="26"/>
+      <c r="J19" s="26"/>
+      <c r="K19" s="29" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="29" t="n">
+    <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="29" t="s">
+      <c r="C20" s="26" t="s">
         <v>207</v>
       </c>
-      <c r="D20" s="29" t="s">
+      <c r="D20" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="29" t="s">
+      <c r="E20" s="26" t="s">
         <v>208</v>
       </c>
-      <c r="F20" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="G20" s="29" t="s">
+      <c r="F20" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="26" t="s">
         <v>209</v>
       </c>
-      <c r="H20" s="29"/>
-      <c r="I20" s="29"/>
-      <c r="J20" s="29"/>
-      <c r="K20" s="31" t="s">
+      <c r="H20" s="26"/>
+      <c r="I20" s="26"/>
+      <c r="J20" s="26"/>
+      <c r="K20" s="28" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="29" t="n">
+    <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B21" s="29" t="s">
+      <c r="B21" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="29" t="s">
+      <c r="C21" s="26" t="s">
         <v>211</v>
       </c>
-      <c r="D21" s="29" t="s">
+      <c r="D21" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="E21" s="29" t="s">
+      <c r="E21" s="26" t="s">
         <v>212</v>
       </c>
-      <c r="F21" s="29" t="s">
+      <c r="F21" s="26" t="s">
         <v>213</v>
       </c>
-      <c r="G21" s="29" t="s">
+      <c r="G21" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="H21" s="29"/>
-      <c r="I21" s="29"/>
-      <c r="J21" s="29"/>
-      <c r="K21" s="30" t="s">
+      <c r="H21" s="26"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="26"/>
+      <c r="K21" s="27" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="29" t="n">
+    <row r="22" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="29" t="s">
+      <c r="C22" s="26" t="s">
         <v>216</v>
       </c>
-      <c r="D22" s="29" t="s">
+      <c r="D22" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="E22" s="29" t="s">
+      <c r="E22" s="26" t="s">
         <v>217</v>
       </c>
-      <c r="F22" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="G22" s="29" t="s">
+      <c r="F22" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" s="26" t="s">
         <v>218</v>
       </c>
-      <c r="H22" s="29"/>
-      <c r="I22" s="29"/>
-      <c r="J22" s="29"/>
-      <c r="K22" s="31" t="s">
+      <c r="H22" s="26"/>
+      <c r="I22" s="26"/>
+      <c r="J22" s="26"/>
+      <c r="K22" s="28" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="29" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B23" s="29" t="s">
+      <c r="B23" s="26" t="s">
         <v>162</v>
       </c>
-      <c r="C23" s="29" t="s">
+      <c r="C23" s="26" t="s">
         <v>219</v>
       </c>
-      <c r="D23" s="29" t="s">
+      <c r="D23" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="29" t="s">
+      <c r="E23" s="26" t="s">
         <v>170</v>
       </c>
-      <c r="F23" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="G23" s="29"/>
-      <c r="H23" s="29"/>
-      <c r="I23" s="29"/>
-      <c r="J23" s="29"/>
-      <c r="K23" s="31" t="s">
+      <c r="F23" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="28" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="29" t="n">
+    <row r="24" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B24" s="29" t="s">
+      <c r="B24" s="26" t="s">
         <v>162</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="26" t="s">
         <v>219</v>
       </c>
-      <c r="D24" s="29" t="s">
+      <c r="D24" s="26" t="s">
         <v>220</v>
       </c>
-      <c r="E24" s="29" t="s">
+      <c r="E24" s="26" t="s">
         <v>221</v>
       </c>
-      <c r="F24" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="29" t="s">
+      <c r="F24" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="26" t="s">
         <v>222</v>
       </c>
-      <c r="H24" s="29"/>
-      <c r="I24" s="29"/>
-      <c r="J24" s="29"/>
-      <c r="K24" s="31" t="s">
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="26"/>
+      <c r="K24" s="28" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="29" t="n">
+      <c r="A25" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B25" s="29" t="s">
+      <c r="B25" s="26" t="s">
         <v>162</v>
       </c>
-      <c r="C25" s="29" t="s">
+      <c r="C25" s="26" t="s">
         <v>223</v>
       </c>
-      <c r="D25" s="29" t="s">
+      <c r="D25" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="29" t="s">
+      <c r="E25" s="26" t="s">
         <v>170</v>
       </c>
-      <c r="F25" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="G25" s="29" t="s">
+      <c r="F25" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="26" t="s">
         <v>224</v>
       </c>
-      <c r="H25" s="29"/>
-      <c r="I25" s="29"/>
-      <c r="J25" s="29"/>
-      <c r="K25" s="31" t="s">
+      <c r="H25" s="26"/>
+      <c r="I25" s="26"/>
+      <c r="J25" s="26"/>
+      <c r="K25" s="28" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="29" t="n">
+    <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B26" s="29" t="s">
+      <c r="B26" s="26" t="s">
         <v>162</v>
       </c>
-      <c r="C26" s="29" t="s">
+      <c r="C26" s="26" t="s">
         <v>223</v>
       </c>
-      <c r="D26" s="29" t="s">
+      <c r="D26" s="26" t="s">
         <v>220</v>
       </c>
-      <c r="E26" s="29" t="s">
+      <c r="E26" s="26" t="s">
         <v>225</v>
       </c>
-      <c r="F26" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="G26" s="29"/>
-      <c r="H26" s="29"/>
-      <c r="I26" s="29"/>
-      <c r="J26" s="29"/>
-      <c r="K26" s="31" t="s">
+      <c r="F26" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="G26" s="26"/>
+      <c r="H26" s="26"/>
+      <c r="I26" s="26"/>
+      <c r="J26" s="26"/>
+      <c r="K26" s="28" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="29" t="n">
+      <c r="A27" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B27" s="29" t="s">
+      <c r="B27" s="26" t="s">
         <v>162</v>
       </c>
-      <c r="C27" s="29" t="s">
+      <c r="C27" s="26" t="s">
         <v>226</v>
       </c>
-      <c r="D27" s="29" t="s">
+      <c r="D27" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="E27" s="29" t="s">
+      <c r="E27" s="26" t="s">
         <v>170</v>
       </c>
-      <c r="F27" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="G27" s="29" t="s">
+      <c r="F27" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" s="26" t="s">
         <v>227</v>
       </c>
-      <c r="H27" s="29"/>
-      <c r="I27" s="29"/>
-      <c r="J27" s="29"/>
-      <c r="K27" s="31" t="s">
+      <c r="H27" s="26"/>
+      <c r="I27" s="26"/>
+      <c r="J27" s="26"/>
+      <c r="K27" s="28" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="29" t="n">
+    <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B28" s="29" t="s">
+      <c r="B28" s="26" t="s">
         <v>162</v>
       </c>
-      <c r="C28" s="29" t="s">
+      <c r="C28" s="26" t="s">
         <v>228</v>
       </c>
-      <c r="D28" s="29" t="s">
+      <c r="D28" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="E28" s="29" t="s">
+      <c r="E28" s="26" t="s">
         <v>229</v>
       </c>
-      <c r="F28" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="G28" s="29" t="s">
+      <c r="F28" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="G28" s="26" t="s">
         <v>230</v>
       </c>
-      <c r="H28" s="29"/>
-      <c r="I28" s="29"/>
-      <c r="J28" s="29"/>
-      <c r="K28" s="31" t="s">
+      <c r="H28" s="26"/>
+      <c r="I28" s="26"/>
+      <c r="J28" s="26"/>
+      <c r="K28" s="28" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="28" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="19" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="33" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="30" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="33" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="30" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="33" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="30" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="33" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="30" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="33" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="30" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="33" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="30" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="33" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="30" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="33" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="30" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="28" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="19" t="s">
         <v>240</v>
       </c>
     </row>
@@ -4948,12 +4947,12 @@
       <c r="K41" s="4"/>
       <c r="L41" s="4"/>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="29"/>
-      <c r="B42" s="29" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="26"/>
+      <c r="B42" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C42" s="29" t="s">
+      <c r="C42" s="26" t="s">
         <v>244</v>
       </c>
       <c r="D42" s="6" t="n">
@@ -4963,12 +4962,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="29"/>
-      <c r="B43" s="29" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="26"/>
+      <c r="B43" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="C43" s="29" t="s">
+      <c r="C43" s="26" t="s">
         <v>244</v>
       </c>
       <c r="D43" s="6" t="n">
@@ -4978,12 +4977,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="29"/>
-      <c r="B44" s="29" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="26"/>
+      <c r="B44" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="C44" s="29" t="s">
+      <c r="C44" s="26" t="s">
         <v>244</v>
       </c>
       <c r="D44" s="6" t="n">
@@ -4993,12 +4992,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="29"/>
-      <c r="B45" s="29" t="s">
+    <row r="45" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="26"/>
+      <c r="B45" s="26" t="s">
         <v>245</v>
       </c>
-      <c r="C45" s="29" t="s">
+      <c r="C45" s="26" t="s">
         <v>244</v>
       </c>
       <c r="D45" s="6" t="n">
@@ -5008,12 +5007,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="29"/>
-      <c r="B46" s="29" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="26"/>
+      <c r="B46" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="C46" s="29" t="s">
+      <c r="C46" s="26" t="s">
         <v>246</v>
       </c>
       <c r="D46" s="6" t="n">
@@ -5023,12 +5022,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="29"/>
-      <c r="B47" s="29" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="26"/>
+      <c r="B47" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="C47" s="29" t="s">
+      <c r="C47" s="26" t="s">
         <v>246</v>
       </c>
       <c r="D47" s="6" t="n">
@@ -5038,12 +5037,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="29"/>
-      <c r="B48" s="29" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="26"/>
+      <c r="B48" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="C48" s="29" t="s">
+      <c r="C48" s="26" t="s">
         <v>246</v>
       </c>
       <c r="D48" s="6" t="n">
@@ -5053,12 +5052,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="29"/>
-      <c r="B49" s="29" t="s">
+    <row r="49" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="26"/>
+      <c r="B49" s="26" t="s">
         <v>247</v>
       </c>
-      <c r="C49" s="29" t="s">
+      <c r="C49" s="26" t="s">
         <v>246</v>
       </c>
       <c r="D49" s="6" t="n">
@@ -5068,60 +5067,60 @@
         <v>95</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="28" t="s">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B50" s="19" t="s">
         <v>248</v>
       </c>
-      <c r="D50" s="34" t="n">
+      <c r="D50" s="31" t="n">
         <f aca="false">2*D42+3*D43+D44+D45</f>
         <v>76</v>
       </c>
-      <c r="E50" s="34" t="n">
+      <c r="E50" s="31" t="n">
         <f aca="false">2*E42+3*E43+E44+E45</f>
         <v>67</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="28" t="s">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B51" s="19" t="s">
         <v>249</v>
       </c>
-      <c r="D51" s="34" t="n">
+      <c r="D51" s="31" t="n">
         <f aca="false">2*D42+3*D43+D44</f>
         <v>46</v>
       </c>
-      <c r="E51" s="34" t="n">
+      <c r="E51" s="31" t="n">
         <f aca="false">2*E42+3*E43+E44</f>
         <v>17</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="28" t="s">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B52" s="19" t="s">
         <v>250</v>
       </c>
-      <c r="D52" s="34" t="n">
+      <c r="D52" s="31" t="n">
         <f aca="false">5*D46+D47+2*D48+D49</f>
         <v>119</v>
       </c>
-      <c r="E52" s="34" t="n">
+      <c r="E52" s="31" t="n">
         <f aca="false">5*E46+E47+2*E48+E49</f>
         <v>121</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="28" t="s">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B53" s="19" t="s">
         <v>251</v>
       </c>
-      <c r="D53" s="34" t="n">
+      <c r="D53" s="31" t="n">
         <f aca="false">5*D46+D47+2*D48</f>
         <v>74</v>
       </c>
-      <c r="E53" s="34" t="n">
+      <c r="E53" s="31" t="n">
         <f aca="false">5*E46+E47+2*E48</f>
         <v>26</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="27" t="s">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="3" t="s">
         <v>252</v>
       </c>
     </row>
@@ -5160,7 +5159,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -5174,434 +5173,460 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="32" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="33" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="34" t="s">
         <v>255</v>
       </c>
-      <c r="B4" s="35" t="s">
+      <c r="B4" s="34" t="s">
         <v>256</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="C4" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="D4" s="35" t="s">
+      <c r="D4" s="34" t="s">
         <v>258</v>
       </c>
-      <c r="E4" s="35" t="s">
+      <c r="E4" s="34" t="s">
         <v>259</v>
       </c>
-      <c r="F4" s="35" t="s">
+      <c r="F4" s="34" t="s">
         <v>260</v>
       </c>
-      <c r="G4" s="35" t="s">
+      <c r="G4" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="H4" s="35" t="s">
+      <c r="H4" s="34" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="36" t="n">
+      <c r="A5" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="26" t="s">
         <v>261</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="26" t="s">
         <v>262</v>
       </c>
-      <c r="E5" s="36" t="s">
+      <c r="E5" s="35" t="s">
         <v>263</v>
       </c>
-      <c r="F5" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" s="29" t="s">
+      <c r="F5" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="26" t="s">
         <v>264</v>
       </c>
-      <c r="H5" s="37" t="s">
+      <c r="H5" s="36" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="36" t="n">
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="26" t="s">
         <v>266</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>262</v>
+      </c>
+      <c r="E6" s="35" t="s">
+        <v>263</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="26" t="s">
+        <v>267</v>
+      </c>
+      <c r="H6" s="36" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="C7" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="D7" s="26" t="s">
         <v>262</v>
       </c>
-      <c r="E6" s="36" t="s">
+      <c r="E7" s="35" t="s">
         <v>263</v>
       </c>
-      <c r="F6" s="36" t="s">
+      <c r="F7" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="29" t="s">
-        <v>267</v>
-      </c>
-      <c r="H6" s="38" t="s">
+      <c r="G7" s="26" t="s">
+        <v>269</v>
+      </c>
+      <c r="H7" s="37" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>268</v>
-      </c>
-      <c r="C7" s="29" t="s">
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>270</v>
+      </c>
+      <c r="C8" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D8" s="26" t="s">
         <v>262</v>
       </c>
-      <c r="E7" s="36" t="s">
+      <c r="E8" s="35" t="s">
         <v>156</v>
       </c>
-      <c r="F7" s="36" t="s">
-        <v>35</v>
-      </c>
-      <c r="G7" s="29" t="s">
-        <v>269</v>
-      </c>
-      <c r="H7" s="38" t="s">
+      <c r="F8" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="26" t="s">
+        <v>271</v>
+      </c>
+      <c r="H8" s="37" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="36" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>270</v>
-      </c>
-      <c r="C8" s="29" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="26" t="s">
+        <v>272</v>
+      </c>
+      <c r="C9" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="D8" s="29" t="s">
-        <v>271</v>
-      </c>
-      <c r="E8" s="36" t="s">
+      <c r="D9" s="26" t="s">
+        <v>273</v>
+      </c>
+      <c r="E9" s="35" t="s">
         <v>263</v>
       </c>
-      <c r="F8" s="36" t="s">
-        <v>26</v>
-      </c>
-      <c r="G8" s="29" t="s">
-        <v>272</v>
-      </c>
-      <c r="H8" s="38" t="s">
+      <c r="F9" s="35" t="s">
+        <v>197</v>
+      </c>
+      <c r="G9" s="26" t="s">
+        <v>274</v>
+      </c>
+      <c r="H9" s="37" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="36" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="29" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="26" t="s">
+        <v>275</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="D10" s="26" t="s">
+        <v>262</v>
+      </c>
+      <c r="E10" s="35" t="s">
+        <v>263</v>
+      </c>
+      <c r="F10" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" s="26" t="s">
+        <v>276</v>
+      </c>
+      <c r="H10" s="37" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="35" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="26" t="s">
+        <v>277</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>278</v>
+      </c>
+      <c r="D11" s="26" t="s">
         <v>273</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="E11" s="35" t="s">
+        <v>263</v>
+      </c>
+      <c r="F11" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="26" t="s">
+        <v>279</v>
+      </c>
+      <c r="H11" s="37" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="26" t="s">
+        <v>280</v>
+      </c>
+      <c r="C12" s="26" t="s">
         <v>244</v>
       </c>
-      <c r="D9" s="29" t="s">
+      <c r="D12" s="26" t="s">
+        <v>281</v>
+      </c>
+      <c r="E12" s="35" t="s">
+        <v>263</v>
+      </c>
+      <c r="F12" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="26" t="s">
+        <v>282</v>
+      </c>
+      <c r="H12" s="38" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="35" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="26" t="s">
+        <v>284</v>
+      </c>
+      <c r="C13" s="26" t="s">
+        <v>162</v>
+      </c>
+      <c r="D13" s="26" t="s">
+        <v>285</v>
+      </c>
+      <c r="E13" s="35" t="s">
+        <v>156</v>
+      </c>
+      <c r="F13" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="G13" s="26" t="s">
+        <v>286</v>
+      </c>
+      <c r="H13" s="37" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="26" t="s">
+        <v>287</v>
+      </c>
+      <c r="C14" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="D14" s="26" t="s">
         <v>262</v>
       </c>
-      <c r="E9" s="36" t="s">
-        <v>263</v>
-      </c>
-      <c r="F9" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" s="29" t="s">
-        <v>274</v>
-      </c>
-      <c r="H9" s="38" t="s">
+      <c r="E14" s="35" t="s">
+        <v>156</v>
+      </c>
+      <c r="F14" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="26" t="s">
+        <v>288</v>
+      </c>
+      <c r="H14" s="37" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="36" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>275</v>
-      </c>
-      <c r="C10" s="29" t="s">
-        <v>276</v>
-      </c>
-      <c r="D10" s="29" t="s">
-        <v>271</v>
-      </c>
-      <c r="E10" s="36" t="s">
-        <v>263</v>
-      </c>
-      <c r="F10" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" s="29" t="s">
-        <v>277</v>
-      </c>
-      <c r="H10" s="38" t="s">
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="35" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="26" t="s">
+        <v>289</v>
+      </c>
+      <c r="C15" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="D15" s="26" t="s">
+        <v>290</v>
+      </c>
+      <c r="E15" s="35" t="s">
+        <v>156</v>
+      </c>
+      <c r="F15" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="G15" s="26" t="s">
+        <v>291</v>
+      </c>
+      <c r="H15" s="37" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="36" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="29" t="s">
-        <v>278</v>
-      </c>
-      <c r="C11" s="29" t="s">
-        <v>244</v>
-      </c>
-      <c r="D11" s="29" t="s">
-        <v>279</v>
-      </c>
-      <c r="E11" s="36" t="s">
-        <v>263</v>
-      </c>
-      <c r="F11" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="G11" s="29" t="s">
-        <v>280</v>
-      </c>
-      <c r="H11" s="39" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="36" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="29" t="s">
-        <v>282</v>
-      </c>
-      <c r="C12" s="29" t="s">
-        <v>162</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>283</v>
-      </c>
-      <c r="E12" s="36" t="s">
+    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="35" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="26" t="s">
+        <v>292</v>
+      </c>
+      <c r="C16" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="D16" s="26" t="s">
+        <v>262</v>
+      </c>
+      <c r="E16" s="35" t="s">
+        <v>293</v>
+      </c>
+      <c r="F16" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="26" t="s">
+        <v>294</v>
+      </c>
+      <c r="H16" s="37" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="35" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="26" t="s">
+        <v>295</v>
+      </c>
+      <c r="C17" s="26" t="s">
+        <v>296</v>
+      </c>
+      <c r="D17" s="26" t="s">
+        <v>262</v>
+      </c>
+      <c r="E17" s="35" t="s">
         <v>156</v>
       </c>
-      <c r="F12" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" s="29" t="s">
-        <v>284</v>
-      </c>
-      <c r="H12" s="38" t="s">
+      <c r="F17" s="35" t="s">
+        <v>297</v>
+      </c>
+      <c r="G17" s="26" t="s">
+        <v>298</v>
+      </c>
+      <c r="H17" s="37" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="36" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="29" t="s">
-        <v>285</v>
-      </c>
-      <c r="C13" s="29" t="s">
-        <v>246</v>
-      </c>
-      <c r="D13" s="29" t="s">
+    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="35" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="26" t="s">
+        <v>299</v>
+      </c>
+      <c r="C18" s="26" t="s">
+        <v>296</v>
+      </c>
+      <c r="D18" s="26" t="s">
         <v>262</v>
       </c>
-      <c r="E13" s="36" t="s">
+      <c r="E18" s="35" t="s">
+        <v>300</v>
+      </c>
+      <c r="F18" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="26" t="s">
+        <v>301</v>
+      </c>
+      <c r="H18" s="37" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="26" t="s">
+        <v>302</v>
+      </c>
+      <c r="C19" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="D19" s="26" t="s">
+        <v>262</v>
+      </c>
+      <c r="E19" s="35" t="s">
         <v>156</v>
       </c>
-      <c r="F13" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="G13" s="29" t="s">
-        <v>286</v>
-      </c>
-      <c r="H13" s="38" t="s">
+      <c r="F19" s="35" t="s">
+        <v>297</v>
+      </c>
+      <c r="G19" s="26" t="s">
+        <v>303</v>
+      </c>
+      <c r="H19" s="37" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="36" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>287</v>
-      </c>
-      <c r="C14" s="29" t="s">
-        <v>246</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>288</v>
-      </c>
-      <c r="E14" s="36" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="35" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="26" t="s">
+        <v>304</v>
+      </c>
+      <c r="C20" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="D20" s="26" t="s">
+        <v>262</v>
+      </c>
+      <c r="E20" s="35" t="s">
         <v>156</v>
       </c>
-      <c r="F14" s="36" t="s">
-        <v>289</v>
-      </c>
-      <c r="G14" s="29" t="s">
-        <v>290</v>
-      </c>
-      <c r="H14" s="38" t="s">
+      <c r="F20" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="26" t="s">
+        <v>305</v>
+      </c>
+      <c r="H20" s="37" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="36" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="29" t="s">
-        <v>291</v>
-      </c>
-      <c r="C15" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>262</v>
-      </c>
-      <c r="E15" s="36" t="s">
-        <v>292</v>
-      </c>
-      <c r="F15" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="G15" s="29" t="s">
-        <v>293</v>
-      </c>
-      <c r="H15" s="38" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="36" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>294</v>
-      </c>
-      <c r="C16" s="29" t="s">
-        <v>295</v>
-      </c>
-      <c r="D16" s="29" t="s">
-        <v>262</v>
-      </c>
-      <c r="E16" s="36" t="s">
-        <v>156</v>
-      </c>
-      <c r="F16" s="36" t="s">
-        <v>296</v>
-      </c>
-      <c r="G16" s="29" t="s">
-        <v>297</v>
-      </c>
-      <c r="H16" s="38" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="36" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="29" t="s">
-        <v>298</v>
-      </c>
-      <c r="C17" s="29" t="s">
-        <v>295</v>
-      </c>
-      <c r="D17" s="29" t="s">
-        <v>262</v>
-      </c>
-      <c r="E17" s="36" t="s">
-        <v>299</v>
-      </c>
-      <c r="F17" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="G17" s="29" t="s">
-        <v>300</v>
-      </c>
-      <c r="H17" s="38" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="36" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>301</v>
-      </c>
-      <c r="C18" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="D18" s="29" t="s">
-        <v>262</v>
-      </c>
-      <c r="E18" s="36" t="s">
-        <v>156</v>
-      </c>
-      <c r="F18" s="36" t="s">
-        <v>296</v>
-      </c>
-      <c r="G18" s="29" t="s">
-        <v>302</v>
-      </c>
-      <c r="H18" s="38" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="36" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="29" t="s">
-        <v>303</v>
-      </c>
-      <c r="C19" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="D19" s="29" t="s">
-        <v>262</v>
-      </c>
-      <c r="E19" s="36" t="s">
-        <v>156</v>
-      </c>
-      <c r="F19" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="G19" s="29" t="s">
-        <v>304</v>
-      </c>
-      <c r="H19" s="38" t="s">
-        <v>171</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:H19"/>
-  <conditionalFormatting sqref="H5:H19">
+  <autoFilter ref="A4:H20"/>
+  <conditionalFormatting sqref="H5:H20">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"Done"</formula>
     </cfRule>
@@ -5616,7 +5641,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H19" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H20" type="list">
       <formula1>"Done,In progress,Not started,Undecided"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5650,139 +5675,139 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="40" t="n">
+      <c r="B5" s="39" t="n">
         <v>0.5</v>
       </c>
-      <c r="C5" s="41" t="n">
+      <c r="C5" s="40" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>315</v>
-      </c>
-      <c r="B6" s="40" t="n">
+        <v>316</v>
+      </c>
+      <c r="B6" s="39" t="n">
         <v>0.2</v>
       </c>
-      <c r="C6" s="41" t="n">
+      <c r="C6" s="40" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>317</v>
-      </c>
-      <c r="B7" s="40" t="n">
+        <v>318</v>
+      </c>
+      <c r="B7" s="39" t="n">
         <v>0.2</v>
       </c>
-      <c r="C7" s="41" t="n">
+      <c r="C7" s="40" t="n">
         <v>1.5</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>319</v>
-      </c>
-      <c r="B8" s="40" t="n">
+        <v>320</v>
+      </c>
+      <c r="B8" s="39" t="n">
         <v>0.1</v>
       </c>
-      <c r="C8" s="41" t="n">
+      <c r="C8" s="40" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="41" t="n">
+      <c r="C9" s="40" t="n">
         <v>2.2</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>325</v>
-      </c>
-      <c r="B11" s="42" t="n">
+        <v>326</v>
+      </c>
+      <c r="B11" s="41" t="n">
         <f aca="false">SUM(B5:B8)</f>
         <v>1</v>
       </c>
@@ -5818,12 +5843,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5831,31 +5856,31 @@
         <v>29</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5865,20 +5890,20 @@
       <c r="B5" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="40" t="n">
+      <c r="C5" s="39" t="n">
         <v>0.25</v>
       </c>
-      <c r="D5" s="41" t="n">
+      <c r="D5" s="40" t="n">
         <v>1.25</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="43" t="n">
+      <c r="F5" s="42" t="n">
         <f aca="false">D5*E5</f>
         <v>2.5</v>
       </c>
-      <c r="G5" s="44" t="n">
+      <c r="G5" s="43" t="n">
         <f aca="false">INDEX(Monsters!$F$5:$F$17,MATCH(A5,Monsters!$A$5:$A$17,0))</f>
         <v>12</v>
       </c>
@@ -5891,7 +5916,7 @@
         <v>60</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5899,22 +5924,22 @@
         <v>37</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="C6" s="40" t="n">
+        <v>335</v>
+      </c>
+      <c r="C6" s="39" t="n">
         <v>0.2</v>
       </c>
-      <c r="D6" s="41" t="n">
+      <c r="D6" s="40" t="n">
         <v>2.25</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="43" t="n">
+      <c r="F6" s="42" t="n">
         <f aca="false">D6*E6</f>
         <v>2.25</v>
       </c>
-      <c r="G6" s="44" t="n">
+      <c r="G6" s="43" t="n">
         <f aca="false">INDEX(Monsters!$F$5:$F$17,MATCH(A6,Monsters!$A$5:$A$17,0))</f>
         <v>10</v>
       </c>
@@ -5927,7 +5952,7 @@
         <v>34</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5935,22 +5960,22 @@
         <v>37</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>336</v>
-      </c>
-      <c r="C7" s="40" t="n">
+        <v>337</v>
+      </c>
+      <c r="C7" s="39" t="n">
         <v>0.15</v>
       </c>
-      <c r="D7" s="41" t="n">
+      <c r="D7" s="40" t="n">
         <v>0.8</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F7" s="43" t="n">
+      <c r="F7" s="42" t="n">
         <f aca="false">D7*E7</f>
         <v>1.6</v>
       </c>
-      <c r="G7" s="44" t="n">
+      <c r="G7" s="43" t="n">
         <f aca="false">INDEX(Monsters!$F$5:$F$17,MATCH(A7,Monsters!$A$5:$A$17,0))</f>
         <v>10</v>
       </c>
@@ -5963,7 +5988,7 @@
         <v>24</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5973,20 +5998,20 @@
       <c r="B8" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="40" t="n">
+      <c r="C8" s="39" t="n">
         <v>0.2</v>
       </c>
-      <c r="D8" s="41" t="n">
+      <c r="D8" s="40" t="n">
         <v>2.5</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="43" t="n">
+      <c r="F8" s="42" t="n">
         <f aca="false">D8*E8</f>
         <v>2.5</v>
       </c>
-      <c r="G8" s="44" t="n">
+      <c r="G8" s="43" t="n">
         <f aca="false">INDEX(Monsters!$F$5:$F$17,MATCH(A8,Monsters!$A$5:$A$17,0))</f>
         <v>34</v>
       </c>
@@ -5999,7 +6024,7 @@
         <v>119</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6007,22 +6032,22 @@
         <v>46</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>339</v>
-      </c>
-      <c r="C9" s="40" t="n">
+        <v>340</v>
+      </c>
+      <c r="C9" s="39" t="n">
         <v>0.15</v>
       </c>
-      <c r="D9" s="41" t="n">
+      <c r="D9" s="40" t="n">
         <v>3</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="43" t="n">
+      <c r="F9" s="42" t="n">
         <f aca="false">D9*E9</f>
         <v>3</v>
       </c>
-      <c r="G9" s="44" t="n">
+      <c r="G9" s="43" t="n">
         <f aca="false">INDEX(Monsters!$F$5:$F$17,MATCH(A9,Monsters!$A$5:$A$17,0))</f>
         <v>42</v>
       </c>
@@ -6035,7 +6060,7 @@
         <v>189</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6043,22 +6068,22 @@
         <v>46</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>341</v>
-      </c>
-      <c r="C10" s="40" t="n">
+        <v>342</v>
+      </c>
+      <c r="C10" s="39" t="n">
         <v>0.15</v>
       </c>
-      <c r="D10" s="41" t="n">
+      <c r="D10" s="40" t="n">
         <v>0.9</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="43" t="n">
+      <c r="F10" s="42" t="n">
         <f aca="false">D10*E10</f>
         <v>1.8</v>
       </c>
-      <c r="G10" s="44" t="n">
+      <c r="G10" s="43" t="n">
         <f aca="false">INDEX(Monsters!$F$5:$F$17,MATCH(A10,Monsters!$A$5:$A$17,0))</f>
         <v>42</v>
       </c>
@@ -6071,7 +6096,7 @@
         <v>113</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6079,22 +6104,22 @@
         <v>46</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>342</v>
-      </c>
-      <c r="C11" s="40" t="n">
+        <v>343</v>
+      </c>
+      <c r="C11" s="39" t="n">
         <v>0.1</v>
       </c>
-      <c r="D11" s="41" t="n">
+      <c r="D11" s="40" t="n">
         <v>1.4</v>
       </c>
       <c r="E11" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="43" t="n">
+      <c r="F11" s="42" t="n">
         <f aca="false">D11*E11</f>
         <v>1.4</v>
       </c>
-      <c r="G11" s="44" t="n">
+      <c r="G11" s="43" t="n">
         <f aca="false">INDEX(Monsters!$F$5:$F$17,MATCH(A11,Monsters!$A$5:$A$17,0))</f>
         <v>42</v>
       </c>
@@ -6107,12 +6132,12 @@
         <v>88</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -6144,12 +6169,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6160,30 +6185,30 @@
         <v>7</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>14</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="45" t="str">
+      <c r="A5" s="44" t="str">
         <f aca="false">Monsters!A5</f>
         <v>Mutated Tadpole</v>
       </c>
-      <c r="B5" s="44" t="n">
+      <c r="B5" s="43" t="n">
         <f aca="false">Monsters!F5</f>
         <v>4</v>
       </c>
@@ -6213,11 +6238,11 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="45" t="str">
+      <c r="A6" s="44" t="str">
         <f aca="false">Monsters!A6</f>
         <v>Mutated Frog</v>
       </c>
-      <c r="B6" s="44" t="n">
+      <c r="B6" s="43" t="n">
         <f aca="false">Monsters!F6</f>
         <v>4</v>
       </c>
@@ -6247,11 +6272,11 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="45" t="str">
+      <c r="A7" s="44" t="str">
         <f aca="false">Monsters!A7</f>
         <v>Mutated Boar</v>
       </c>
-      <c r="B7" s="44" t="n">
+      <c r="B7" s="43" t="n">
         <f aca="false">Monsters!F7</f>
         <v>12</v>
       </c>
@@ -6281,11 +6306,11 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="46" t="str">
+      <c r="A8" s="45" t="str">
         <f aca="false">Monsters!A8</f>
         <v>Mutated Cheetah</v>
       </c>
-      <c r="B8" s="47" t="n">
+      <c r="B8" s="46" t="n">
         <f aca="false">Monsters!F8</f>
         <v>12</v>
       </c>
@@ -6315,11 +6340,11 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="45" t="str">
+      <c r="A9" s="44" t="str">
         <f aca="false">Monsters!A9</f>
         <v>Security Drone</v>
       </c>
-      <c r="B9" s="44" t="n">
+      <c r="B9" s="43" t="n">
         <f aca="false">Monsters!F9</f>
         <v>5</v>
       </c>
@@ -6349,11 +6374,11 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="45" t="str">
+      <c r="A10" s="44" t="str">
         <f aca="false">Monsters!A10</f>
         <v>Maintenance Bot</v>
       </c>
-      <c r="B10" s="44" t="n">
+      <c r="B10" s="43" t="n">
         <f aca="false">Monsters!F10</f>
         <v>8</v>
       </c>
@@ -6383,11 +6408,11 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="45" t="str">
+      <c r="A11" s="44" t="str">
         <f aca="false">Monsters!A11</f>
         <v>Sentry Turret</v>
       </c>
-      <c r="B11" s="44" t="n">
+      <c r="B11" s="43" t="n">
         <f aca="false">Monsters!F11</f>
         <v>9</v>
       </c>
@@ -6417,11 +6442,11 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="46" t="str">
+      <c r="A12" s="45" t="str">
         <f aca="false">Monsters!A12</f>
         <v>Rogue Overseer</v>
       </c>
-      <c r="B12" s="47" t="n">
+      <c r="B12" s="46" t="n">
         <f aca="false">Monsters!F12</f>
         <v>10</v>
       </c>
@@ -6451,11 +6476,11 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="45" t="str">
+      <c r="A13" s="44" t="str">
         <f aca="false">Monsters!A13</f>
         <v>Rift Wisp</v>
       </c>
-      <c r="B13" s="44" t="n">
+      <c r="B13" s="43" t="n">
         <f aca="false">Monsters!F13</f>
         <v>18</v>
       </c>
@@ -6485,11 +6510,11 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="45" t="str">
+      <c r="A14" s="44" t="str">
         <f aca="false">Monsters!A14</f>
         <v>Rift Knight</v>
       </c>
-      <c r="B14" s="44" t="n">
+      <c r="B14" s="43" t="n">
         <f aca="false">Monsters!F14</f>
         <v>32</v>
       </c>
@@ -6519,11 +6544,11 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="45" t="str">
+      <c r="A15" s="44" t="str">
         <f aca="false">Monsters!A15</f>
         <v>Rift Stalker</v>
       </c>
-      <c r="B15" s="44" t="n">
+      <c r="B15" s="43" t="n">
         <f aca="false">Monsters!F15</f>
         <v>35</v>
       </c>
@@ -6553,11 +6578,11 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="46" t="str">
+      <c r="A16" s="45" t="str">
         <f aca="false">Monsters!A16</f>
         <v>Rift Warden</v>
       </c>
-      <c r="B16" s="47" t="n">
+      <c r="B16" s="46" t="n">
         <f aca="false">Monsters!F16</f>
         <v>34</v>
       </c>
@@ -6587,11 +6612,11 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="46" t="str">
+      <c r="A17" s="45" t="str">
         <f aca="false">Monsters!A17</f>
         <v>Hollow Colossus</v>
       </c>
-      <c r="B17" s="47" t="n">
+      <c r="B17" s="46" t="n">
         <f aca="false">Monsters!F17</f>
         <v>42</v>
       </c>
@@ -6649,633 +6674,633 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="35" t="s">
-        <v>354</v>
-      </c>
-      <c r="B4" s="35" t="s">
+      <c r="A4" s="34" t="s">
+        <v>355</v>
+      </c>
+      <c r="B4" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="C4" s="35" t="s">
-        <v>355</v>
-      </c>
-      <c r="D4" s="35" t="s">
+      <c r="C4" s="34" t="s">
         <v>356</v>
       </c>
-      <c r="E4" s="35" t="s">
+      <c r="D4" s="34" t="s">
         <v>357</v>
       </c>
-      <c r="F4" s="35" t="s">
+      <c r="E4" s="34" t="s">
         <v>358</v>
       </c>
-      <c r="G4" s="35" t="s">
+      <c r="F4" s="34" t="s">
         <v>359</v>
       </c>
+      <c r="G4" s="34" t="s">
+        <v>360</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
-        <v>360</v>
-      </c>
-      <c r="B5" s="29" t="s">
+      <c r="A5" s="26" t="s">
         <v>361</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="B5" s="26" t="s">
         <v>362</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="C5" s="26" t="s">
         <v>363</v>
       </c>
-      <c r="E5" s="29" t="s">
+      <c r="D5" s="26" t="s">
         <v>364</v>
       </c>
-      <c r="F5" s="29" t="s">
+      <c r="E5" s="26" t="s">
         <v>365</v>
       </c>
-      <c r="G5" s="29" t="s">
+      <c r="F5" s="26" t="s">
         <v>366</v>
       </c>
+      <c r="G5" s="26" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29" t="s">
-        <v>360</v>
-      </c>
-      <c r="B6" s="29" t="s">
+      <c r="A6" s="26" t="s">
+        <v>361</v>
+      </c>
+      <c r="B6" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="26" t="s">
+        <v>368</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>369</v>
+      </c>
+      <c r="E6" s="26" t="s">
+        <v>370</v>
+      </c>
+      <c r="F6" s="26" t="s">
+        <v>371</v>
+      </c>
+      <c r="G6" s="26" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="26" t="s">
+        <v>373</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>374</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>375</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="26" t="s">
+        <v>376</v>
+      </c>
+      <c r="F7" s="26" t="s">
+        <v>377</v>
+      </c>
+      <c r="G7" s="26" t="s">
         <v>367</v>
       </c>
-      <c r="D6" s="29" t="s">
-        <v>368</v>
-      </c>
-      <c r="E6" s="29" t="s">
-        <v>369</v>
-      </c>
-      <c r="F6" s="29" t="s">
-        <v>370</v>
-      </c>
-      <c r="G6" s="29" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="s">
-        <v>372</v>
-      </c>
-      <c r="B7" s="29" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="26" t="s">
         <v>373</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="B8" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>378</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="26" t="s">
+        <v>379</v>
+      </c>
+      <c r="F8" s="26" t="s">
+        <v>380</v>
+      </c>
+      <c r="G8" s="26" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="26" t="s">
+        <v>373</v>
+      </c>
+      <c r="B9" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>381</v>
+      </c>
+      <c r="D9" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="26" t="s">
+        <v>382</v>
+      </c>
+      <c r="F9" s="26" t="s">
+        <v>383</v>
+      </c>
+      <c r="G9" s="26" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B10" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>385</v>
+      </c>
+      <c r="D10" s="26" t="s">
+        <v>386</v>
+      </c>
+      <c r="E10" s="26" t="s">
+        <v>387</v>
+      </c>
+      <c r="F10" s="26" t="s">
+        <v>388</v>
+      </c>
+      <c r="G10" s="26" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B11" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>390</v>
+      </c>
+      <c r="D11" s="26" t="s">
+        <v>391</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>392</v>
+      </c>
+      <c r="F11" s="26" t="s">
+        <v>393</v>
+      </c>
+      <c r="G11" s="26" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B12" s="26" t="s">
+        <v>244</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>394</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>395</v>
+      </c>
+      <c r="E12" s="26" t="s">
+        <v>396</v>
+      </c>
+      <c r="F12" s="26" t="s">
+        <v>397</v>
+      </c>
+      <c r="G12" s="26" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B13" s="26" t="s">
         <v>374</v>
       </c>
-      <c r="D7" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="29" t="s">
+      <c r="C13" s="26" t="s">
         <v>375</v>
       </c>
-      <c r="F7" s="29" t="s">
+      <c r="D13" s="26" t="s">
         <v>376</v>
       </c>
-      <c r="G7" s="29" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29" t="s">
-        <v>372</v>
-      </c>
-      <c r="B8" s="29" t="s">
+      <c r="E13" s="26" t="s">
+        <v>398</v>
+      </c>
+      <c r="F13" s="26" t="s">
+        <v>399</v>
+      </c>
+      <c r="G13" s="26" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B14" s="26" t="s">
+        <v>400</v>
+      </c>
+      <c r="C14" s="26" t="s">
+        <v>401</v>
+      </c>
+      <c r="D14" s="26" t="s">
+        <v>402</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>403</v>
+      </c>
+      <c r="F14" s="26" t="s">
+        <v>404</v>
+      </c>
+      <c r="G14" s="26" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B15" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="C8" s="29" t="s">
-        <v>377</v>
-      </c>
-      <c r="D8" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8" s="29" t="s">
-        <v>378</v>
-      </c>
-      <c r="F8" s="29" t="s">
-        <v>379</v>
-      </c>
-      <c r="G8" s="29" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="s">
-        <v>372</v>
-      </c>
-      <c r="B9" s="29" t="s">
+      <c r="C15" s="26" t="s">
+        <v>405</v>
+      </c>
+      <c r="D15" s="26" t="s">
+        <v>406</v>
+      </c>
+      <c r="E15" s="26" t="s">
+        <v>407</v>
+      </c>
+      <c r="F15" s="26" t="s">
+        <v>408</v>
+      </c>
+      <c r="G15" s="26" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B16" s="26" t="s">
         <v>244</v>
       </c>
-      <c r="C9" s="29" t="s">
-        <v>380</v>
-      </c>
-      <c r="D9" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="29" t="s">
-        <v>381</v>
-      </c>
-      <c r="F9" s="29" t="s">
-        <v>382</v>
-      </c>
-      <c r="G9" s="29" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B10" s="29" t="s">
+      <c r="C16" s="26" t="s">
+        <v>409</v>
+      </c>
+      <c r="D16" s="26" t="s">
+        <v>410</v>
+      </c>
+      <c r="E16" s="26" t="s">
+        <v>411</v>
+      </c>
+      <c r="F16" s="26" t="s">
+        <v>412</v>
+      </c>
+      <c r="G16" s="26" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B17" s="26" t="s">
+        <v>362</v>
+      </c>
+      <c r="C17" s="26" t="s">
+        <v>414</v>
+      </c>
+      <c r="D17" s="26" t="s">
+        <v>415</v>
+      </c>
+      <c r="E17" s="26" t="s">
+        <v>416</v>
+      </c>
+      <c r="F17" s="26" t="s">
+        <v>417</v>
+      </c>
+      <c r="G17" s="26" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B18" s="26" t="s">
+        <v>362</v>
+      </c>
+      <c r="C18" s="26" t="s">
+        <v>418</v>
+      </c>
+      <c r="D18" s="26" t="s">
+        <v>419</v>
+      </c>
+      <c r="E18" s="26" t="s">
+        <v>420</v>
+      </c>
+      <c r="F18" s="26" t="s">
+        <v>421</v>
+      </c>
+      <c r="G18" s="26" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B19" s="26" t="s">
         <v>244</v>
       </c>
-      <c r="C10" s="29" t="s">
+      <c r="C19" s="26" t="s">
+        <v>423</v>
+      </c>
+      <c r="D19" s="26" t="s">
+        <v>424</v>
+      </c>
+      <c r="E19" s="26" t="s">
+        <v>425</v>
+      </c>
+      <c r="F19" s="26" t="s">
+        <v>426</v>
+      </c>
+      <c r="G19" s="26" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="26" t="s">
         <v>384</v>
       </c>
-      <c r="D10" s="29" t="s">
-        <v>385</v>
-      </c>
-      <c r="E10" s="29" t="s">
-        <v>386</v>
-      </c>
-      <c r="F10" s="29" t="s">
-        <v>387</v>
-      </c>
-      <c r="G10" s="29" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B11" s="29" t="s">
+      <c r="B20" s="26" t="s">
         <v>244</v>
       </c>
-      <c r="C11" s="29" t="s">
+      <c r="C20" s="26" t="s">
+        <v>428</v>
+      </c>
+      <c r="D20" s="26" t="s">
+        <v>429</v>
+      </c>
+      <c r="E20" s="26" t="s">
+        <v>430</v>
+      </c>
+      <c r="F20" s="26" t="s">
+        <v>431</v>
+      </c>
+      <c r="G20" s="26" t="s">
         <v>389</v>
       </c>
-      <c r="D11" s="29" t="s">
-        <v>390</v>
-      </c>
-      <c r="E11" s="29" t="s">
-        <v>391</v>
-      </c>
-      <c r="F11" s="29" t="s">
-        <v>392</v>
-      </c>
-      <c r="G11" s="29" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B12" s="29" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B21" s="26" t="s">
         <v>244</v>
       </c>
-      <c r="C12" s="29" t="s">
-        <v>393</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>394</v>
-      </c>
-      <c r="E12" s="29" t="s">
-        <v>395</v>
-      </c>
-      <c r="F12" s="29" t="s">
-        <v>396</v>
-      </c>
-      <c r="G12" s="29" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B13" s="29" t="s">
-        <v>373</v>
-      </c>
-      <c r="C13" s="29" t="s">
-        <v>374</v>
-      </c>
-      <c r="D13" s="29" t="s">
-        <v>375</v>
-      </c>
-      <c r="E13" s="29" t="s">
-        <v>397</v>
-      </c>
-      <c r="F13" s="29" t="s">
-        <v>398</v>
-      </c>
-      <c r="G13" s="29" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>399</v>
-      </c>
-      <c r="C14" s="29" t="s">
-        <v>400</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>401</v>
-      </c>
-      <c r="E14" s="29" t="s">
-        <v>402</v>
-      </c>
-      <c r="F14" s="29" t="s">
-        <v>403</v>
-      </c>
-      <c r="G14" s="29" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B15" s="29" t="s">
+      <c r="C21" s="26" t="s">
+        <v>432</v>
+      </c>
+      <c r="D21" s="26" t="s">
+        <v>433</v>
+      </c>
+      <c r="E21" s="26" t="s">
+        <v>434</v>
+      </c>
+      <c r="F21" s="26" t="s">
+        <v>435</v>
+      </c>
+      <c r="G21" s="26" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B22" s="26" t="s">
+        <v>183</v>
+      </c>
+      <c r="C22" s="26" t="s">
+        <v>436</v>
+      </c>
+      <c r="D22" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="E22" s="26" t="s">
+        <v>437</v>
+      </c>
+      <c r="F22" s="26" t="s">
+        <v>438</v>
+      </c>
+      <c r="G22" s="26" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B23" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="C15" s="29" t="s">
-        <v>404</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>405</v>
-      </c>
-      <c r="E15" s="29" t="s">
-        <v>406</v>
-      </c>
-      <c r="F15" s="29" t="s">
-        <v>407</v>
-      </c>
-      <c r="G15" s="29" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B16" s="29" t="s">
+      <c r="C23" s="26" t="s">
+        <v>439</v>
+      </c>
+      <c r="D23" s="26" t="s">
+        <v>440</v>
+      </c>
+      <c r="E23" s="26" t="s">
+        <v>195</v>
+      </c>
+      <c r="F23" s="26" t="s">
+        <v>441</v>
+      </c>
+      <c r="G23" s="26" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B24" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="C24" s="26" t="s">
+        <v>442</v>
+      </c>
+      <c r="D24" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="E24" s="26" t="s">
+        <v>443</v>
+      </c>
+      <c r="F24" s="26" t="s">
+        <v>444</v>
+      </c>
+      <c r="G24" s="26" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B25" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="C25" s="26" t="s">
+        <v>445</v>
+      </c>
+      <c r="D25" s="26" t="s">
+        <v>429</v>
+      </c>
+      <c r="E25" s="26" t="s">
+        <v>446</v>
+      </c>
+      <c r="F25" s="26" t="s">
+        <v>447</v>
+      </c>
+      <c r="G25" s="26" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B26" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="C26" s="26" t="s">
+        <v>448</v>
+      </c>
+      <c r="D26" s="26" t="s">
+        <v>449</v>
+      </c>
+      <c r="E26" s="26" t="s">
+        <v>450</v>
+      </c>
+      <c r="F26" s="26" t="s">
+        <v>451</v>
+      </c>
+      <c r="G26" s="26" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B27" s="26" t="s">
+        <v>246</v>
+      </c>
+      <c r="C27" s="26" t="s">
+        <v>452</v>
+      </c>
+      <c r="D27" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="E27" s="26" t="s">
+        <v>453</v>
+      </c>
+      <c r="F27" s="26" t="s">
+        <v>454</v>
+      </c>
+      <c r="G27" s="26" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B28" s="26" t="s">
+        <v>455</v>
+      </c>
+      <c r="C28" s="26" t="s">
+        <v>456</v>
+      </c>
+      <c r="D28" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="E28" s="26" t="s">
+        <v>457</v>
+      </c>
+      <c r="F28" s="26" t="s">
+        <v>458</v>
+      </c>
+      <c r="G28" s="26" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="B29" s="26" t="s">
+        <v>459</v>
+      </c>
+      <c r="C29" s="26" t="s">
+        <v>460</v>
+      </c>
+      <c r="D29" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="E29" s="26" t="s">
+        <v>461</v>
+      </c>
+      <c r="F29" s="26" t="s">
+        <v>462</v>
+      </c>
+      <c r="G29" s="26" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="26" t="s">
+        <v>463</v>
+      </c>
+      <c r="B30" s="26" t="s">
         <v>244</v>
       </c>
-      <c r="C16" s="29" t="s">
-        <v>408</v>
-      </c>
-      <c r="D16" s="29" t="s">
-        <v>409</v>
-      </c>
-      <c r="E16" s="29" t="s">
-        <v>410</v>
-      </c>
-      <c r="F16" s="29" t="s">
-        <v>411</v>
-      </c>
-      <c r="G16" s="29" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B17" s="29" t="s">
-        <v>361</v>
-      </c>
-      <c r="C17" s="29" t="s">
-        <v>413</v>
-      </c>
-      <c r="D17" s="29" t="s">
-        <v>414</v>
-      </c>
-      <c r="E17" s="29" t="s">
-        <v>415</v>
-      </c>
-      <c r="F17" s="29" t="s">
-        <v>416</v>
-      </c>
-      <c r="G17" s="29" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>361</v>
-      </c>
-      <c r="C18" s="29" t="s">
-        <v>417</v>
-      </c>
-      <c r="D18" s="29" t="s">
-        <v>418</v>
-      </c>
-      <c r="E18" s="29" t="s">
-        <v>419</v>
-      </c>
-      <c r="F18" s="29" t="s">
-        <v>420</v>
-      </c>
-      <c r="G18" s="29" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B19" s="29" t="s">
-        <v>244</v>
-      </c>
-      <c r="C19" s="29" t="s">
-        <v>422</v>
-      </c>
-      <c r="D19" s="29" t="s">
-        <v>423</v>
-      </c>
-      <c r="E19" s="29" t="s">
-        <v>424</v>
-      </c>
-      <c r="F19" s="29" t="s">
-        <v>425</v>
-      </c>
-      <c r="G19" s="29" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B20" s="29" t="s">
-        <v>244</v>
-      </c>
-      <c r="C20" s="29" t="s">
-        <v>427</v>
-      </c>
-      <c r="D20" s="29" t="s">
-        <v>428</v>
-      </c>
-      <c r="E20" s="29" t="s">
-        <v>429</v>
-      </c>
-      <c r="F20" s="29" t="s">
-        <v>430</v>
-      </c>
-      <c r="G20" s="29" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B21" s="29" t="s">
-        <v>244</v>
-      </c>
-      <c r="C21" s="29" t="s">
-        <v>431</v>
-      </c>
-      <c r="D21" s="29" t="s">
-        <v>432</v>
-      </c>
-      <c r="E21" s="29" t="s">
-        <v>433</v>
-      </c>
-      <c r="F21" s="29" t="s">
-        <v>434</v>
-      </c>
-      <c r="G21" s="29" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B22" s="29" t="s">
-        <v>183</v>
-      </c>
-      <c r="C22" s="29" t="s">
-        <v>435</v>
-      </c>
-      <c r="D22" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="E22" s="29" t="s">
-        <v>436</v>
-      </c>
-      <c r="F22" s="29" t="s">
-        <v>437</v>
-      </c>
-      <c r="G22" s="29" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B23" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="C23" s="29" t="s">
-        <v>438</v>
-      </c>
-      <c r="D23" s="29" t="s">
-        <v>439</v>
-      </c>
-      <c r="E23" s="29" t="s">
-        <v>195</v>
-      </c>
-      <c r="F23" s="29" t="s">
-        <v>440</v>
-      </c>
-      <c r="G23" s="29" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B24" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="C24" s="29" t="s">
-        <v>441</v>
-      </c>
-      <c r="D24" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="E24" s="29" t="s">
-        <v>442</v>
-      </c>
-      <c r="F24" s="29" t="s">
-        <v>443</v>
-      </c>
-      <c r="G24" s="29" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B25" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="C25" s="29" t="s">
-        <v>444</v>
-      </c>
-      <c r="D25" s="29" t="s">
-        <v>428</v>
-      </c>
-      <c r="E25" s="29" t="s">
-        <v>445</v>
-      </c>
-      <c r="F25" s="29" t="s">
-        <v>446</v>
-      </c>
-      <c r="G25" s="29" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B26" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="C26" s="29" t="s">
-        <v>447</v>
-      </c>
-      <c r="D26" s="29" t="s">
-        <v>448</v>
-      </c>
-      <c r="E26" s="29" t="s">
-        <v>449</v>
-      </c>
-      <c r="F26" s="29" t="s">
-        <v>450</v>
-      </c>
-      <c r="G26" s="29" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B27" s="29" t="s">
-        <v>246</v>
-      </c>
-      <c r="C27" s="29" t="s">
-        <v>451</v>
-      </c>
-      <c r="D27" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="E27" s="29" t="s">
-        <v>452</v>
-      </c>
-      <c r="F27" s="29" t="s">
-        <v>453</v>
-      </c>
-      <c r="G27" s="29" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B28" s="29" t="s">
-        <v>454</v>
-      </c>
-      <c r="C28" s="29" t="s">
-        <v>455</v>
-      </c>
-      <c r="D28" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="E28" s="29" t="s">
-        <v>456</v>
-      </c>
-      <c r="F28" s="29" t="s">
-        <v>457</v>
-      </c>
-      <c r="G28" s="29" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B29" s="29" t="s">
-        <v>458</v>
-      </c>
-      <c r="C29" s="29" t="s">
-        <v>459</v>
-      </c>
-      <c r="D29" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="E29" s="29" t="s">
-        <v>460</v>
-      </c>
-      <c r="F29" s="29" t="s">
-        <v>461</v>
-      </c>
-      <c r="G29" s="29" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="29" t="s">
-        <v>462</v>
-      </c>
-      <c r="B30" s="29" t="s">
-        <v>244</v>
-      </c>
-      <c r="C30" s="29" t="s">
-        <v>463</v>
-      </c>
-      <c r="D30" s="29" t="s">
+      <c r="C30" s="26" t="s">
         <v>464</v>
       </c>
-      <c r="E30" s="29" t="s">
+      <c r="D30" s="26" t="s">
         <v>465</v>
       </c>
-      <c r="F30" s="29" t="s">
+      <c r="E30" s="26" t="s">
         <v>466</v>
       </c>
-      <c r="G30" s="29" t="s">
-        <v>388</v>
+      <c r="F30" s="26" t="s">
+        <v>467</v>
+      </c>
+      <c r="G30" s="26" t="s">
+        <v>389</v>
       </c>
     </row>
   </sheetData>

</xml_diff>